<commit_message>
Extend 45-day cluster sheet with redistribution items
- Include all selling SKUs with 45-day need >=10 in cluster breakdown
- Distinguish ДОКУПКА (short on 45-day cover) vs ПЕРЕРАСПРЕДЕЛЕНИЕ
  (volume sufficient but stock sits in Moscow — spread to clusters)
- PDRN and similar now shown with target cluster placement

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0153XBqtvJYtRAKHdw3RmMsz
</commit_message>
<xml_diff>
--- a/outputs/ozon_fbo_plan/ozon_supply_plan_45d_all_2026-10-08.xlsx
+++ b/outputs/ozon_fbo_plan/ozon_supply_plan_45d_all_2026-10-08.xlsx
@@ -108,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -125,6 +125,7 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2432,7 +2433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E99"/>
+  <dimension ref="A1:E163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -2445,7 +2446,7 @@
     <row r="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>РАЗБИВКА ПОСТАВКИ ПО КЛАСТЕРАМ (доля спроса кластера; где нет данных — общая доля магазина)</t>
+          <t>РАЗБИВКА ПО КЛАСТЕРАМ: ДОКУПКА (не хватает на 45 дн) + ПЕРЕРАСПРЕДЕЛЕНИЕ (объёма хватает, но лежит в Москве)</t>
         </is>
       </c>
     </row>
@@ -2479,7 +2480,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>celimax Тонер кремовый увлажняющий с мол</t>
+          <t>celimax Тонер кремовый увлажняющий с мол — ДОКУПКА (не хватает на 45 дн)</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -2788,7 +2789,7 @@
       <c r="A20" s="13" t="inlineStr"/>
       <c r="B20" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ИТОГО</t>
+          <t xml:space="preserve"> ИТОГО докупка</t>
         </is>
       </c>
       <c r="C20" s="13" t="inlineStr"/>
@@ -2800,7 +2801,7 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>celimax Крем-бустер для лица с ретинолом</t>
+          <t>celimax Крем-бустер для лица с ретинолом — ДОКУПКА (не хватает на 45 дн)</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -3071,7 +3072,7 @@
       <c r="A36" s="13" t="inlineStr"/>
       <c r="B36" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ИТОГО</t>
+          <t xml:space="preserve"> ИТОГО докупка</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr"/>
@@ -3083,7 +3084,7 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Round Lab Очищающая пенка для лица с мор</t>
+          <t>Round Lab Очищающая пенка для лица с мор — ДОКУПКА (не хватает на 45 дн)</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -3411,7 +3412,7 @@
       <c r="A55" s="13" t="inlineStr"/>
       <c r="B55" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ИТОГО</t>
+          <t xml:space="preserve"> ИТОГО докупка</t>
         </is>
       </c>
       <c r="C55" s="13" t="inlineStr"/>
@@ -3423,7 +3424,7 @@
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>celimax Лифтинг-сыворотка для лица с рет</t>
+          <t>celimax Лифтинг-сыворотка для лица с рет — ДОКУПКА (не хватает на 45 дн)</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
@@ -3694,7 +3695,7 @@
       <c r="A71" s="13" t="inlineStr"/>
       <c r="B71" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ИТОГО</t>
+          <t xml:space="preserve"> ИТОГО докупка</t>
         </is>
       </c>
       <c r="C71" s="13" t="inlineStr"/>
@@ -3706,7 +3707,7 @@
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>Round Lab Тонер с морской водой увлажняю</t>
+          <t>Round Lab Тонер с морской водой увлажняю — ДОКУПКА (не хватает на 45 дн)</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
@@ -3958,7 +3959,7 @@
       <c r="A86" s="13" t="inlineStr"/>
       <c r="B86" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ИТОГО</t>
+          <t xml:space="preserve"> ИТОГО докупка</t>
         </is>
       </c>
       <c r="C86" s="13" t="inlineStr"/>
@@ -3970,7 +3971,7 @@
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>Крем для восстановления барьера лица</t>
+          <t>PDRN сыворотка для лица VT Essence 100 V — ПЕРЕРАСПРЕДЕЛЕНИЕ (объёма хватает, развезти из Москвы)</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
@@ -3979,10 +3980,10 @@
         </is>
       </c>
       <c r="C88" s="3" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D88" s="3" t="n">
-        <v>21</v>
+        <v>220</v>
       </c>
       <c r="E88" s="11" t="inlineStr">
         <is>
@@ -3994,14 +3995,14 @@
       <c r="A89" s="3" t="inlineStr"/>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>Дальний Восток</t>
+          <t>Санкт-Петербург и СЗО</t>
         </is>
       </c>
       <c r="C89" s="3" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D89" s="3" t="n">
-        <v>8</v>
+        <v>55</v>
       </c>
       <c r="E89" s="12" t="inlineStr">
         <is>
@@ -4013,14 +4014,14 @@
       <c r="A90" s="3" t="inlineStr"/>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>Санкт-Петербург и СЗО</t>
+          <t>Ростов</t>
         </is>
       </c>
       <c r="C90" s="3" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D90" s="3" t="n">
-        <v>8</v>
+        <v>55</v>
       </c>
       <c r="E90" s="12" t="inlineStr">
         <is>
@@ -4032,14 +4033,14 @@
       <c r="A91" s="3" t="inlineStr"/>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>Ростов</t>
+          <t>Краснодар</t>
         </is>
       </c>
       <c r="C91" s="3" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="D91" s="3" t="n">
-        <v>8</v>
+        <v>49</v>
       </c>
       <c r="E91" s="12" t="inlineStr">
         <is>
@@ -4051,14 +4052,14 @@
       <c r="A92" s="3" t="inlineStr"/>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>Воронеж</t>
+          <t>Новосибирск</t>
         </is>
       </c>
       <c r="C92" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D92" s="3" t="n">
-        <v>3</v>
+        <v>37</v>
       </c>
       <c r="E92" s="12" t="inlineStr">
         <is>
@@ -4070,14 +4071,14 @@
       <c r="A93" s="3" t="inlineStr"/>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>Ярославль</t>
+          <t>Дальний Восток</t>
         </is>
       </c>
       <c r="C93" s="3" t="n">
         <v>5</v>
       </c>
       <c r="D93" s="3" t="n">
-        <v>3</v>
+        <v>31</v>
       </c>
       <c r="E93" s="12" t="inlineStr">
         <is>
@@ -4089,88 +4090,1115 @@
       <c r="A94" s="3" t="inlineStr"/>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>Новосибирск</t>
+          <t>Казань</t>
         </is>
       </c>
       <c r="C94" s="3" t="n">
         <v>5</v>
       </c>
       <c r="D94" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="E94" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="3" t="inlineStr"/>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>Калининград</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E94" s="12" t="inlineStr">
-        <is>
-          <t>грузить</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="13" t="inlineStr"/>
-      <c r="B95" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> ИТОГО</t>
-        </is>
-      </c>
-      <c r="C95" s="13" t="inlineStr"/>
-      <c r="D95" s="13" t="n">
+      <c r="D95" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="E95" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr"/>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>Самара</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D96" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="E96" s="5" t="inlineStr">
+        <is>
+          <t>СКЛАД СГОРЕЛ → соседний</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="3" t="inlineStr"/>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>Махачкала</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D97" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="E97" s="5" t="inlineStr">
+        <is>
+          <t>СКЛАД СГОРЕЛ → соседний</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="14" t="inlineStr"/>
+      <c r="B98" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> ИТОГО (перераспределение)</t>
+        </is>
+      </c>
+      <c r="C98" s="14" t="inlineStr"/>
+      <c r="D98" s="14" t="n">
+        <v>630</v>
+      </c>
+      <c r="E98" s="14" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="3" t="inlineStr">
+        <is>
+          <t>Сыворотка с микроиглами для лица VT Reed — ПЕРЕРАСПРЕДЕЛЕНИЕ (объёма хватает, развезти из Москвы)</t>
+        </is>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>Ростов</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="D100" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="E100" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="3" t="inlineStr"/>
+      <c r="B101" s="3" t="inlineStr">
+        <is>
+          <t>Москва, МО и Дальние регионы</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="D101" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="E101" s="11" t="inlineStr">
+        <is>
+          <t>база, не перегружать</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="3" t="inlineStr"/>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>Санкт-Петербург и СЗО</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="D102" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E102" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="3" t="inlineStr"/>
+      <c r="B103" s="3" t="inlineStr">
+        <is>
+          <t>Беларусь</t>
+        </is>
+      </c>
+      <c r="C103" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D103" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E103" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="3" t="inlineStr"/>
+      <c r="B104" s="3" t="inlineStr">
+        <is>
+          <t>Дальний Восток</t>
+        </is>
+      </c>
+      <c r="C104" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D104" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E104" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="3" t="inlineStr"/>
+      <c r="B105" s="3" t="inlineStr">
+        <is>
+          <t>Уфа</t>
+        </is>
+      </c>
+      <c r="C105" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D105" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E105" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="3" t="inlineStr"/>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>Невинномысск</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D106" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E106" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="14" t="inlineStr"/>
+      <c r="B107" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> ИТОГО (перераспределение)</t>
+        </is>
+      </c>
+      <c r="C107" s="14" t="inlineStr"/>
+      <c r="D107" s="14" t="n">
+        <v>90</v>
+      </c>
+      <c r="E107" s="14" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="3" t="inlineStr">
+        <is>
+          <t>Крем для восстановления барьера лица — ДОКУПКА (не хватает на 45 дн)</t>
+        </is>
+      </c>
+      <c r="B109" s="3" t="inlineStr">
+        <is>
+          <t>Москва, МО и Дальние регионы</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="D109" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="E109" s="11" t="inlineStr">
+        <is>
+          <t>база, не перегружать</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="3" t="inlineStr"/>
+      <c r="B110" s="3" t="inlineStr">
+        <is>
+          <t>Дальний Восток</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="D110" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E110" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="3" t="inlineStr"/>
+      <c r="B111" s="3" t="inlineStr">
+        <is>
+          <t>Санкт-Петербург и СЗО</t>
+        </is>
+      </c>
+      <c r="C111" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="D111" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E111" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="3" t="inlineStr"/>
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t>Ростов</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="D112" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E112" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="3" t="inlineStr"/>
+      <c r="B113" s="3" t="inlineStr">
+        <is>
+          <t>Воронеж</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D113" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E113" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="3" t="inlineStr"/>
+      <c r="B114" s="3" t="inlineStr">
+        <is>
+          <t>Ярославль</t>
+        </is>
+      </c>
+      <c r="C114" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D114" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E114" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="3" t="inlineStr"/>
+      <c r="B115" s="3" t="inlineStr">
+        <is>
+          <t>Новосибирск</t>
+        </is>
+      </c>
+      <c r="C115" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D115" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E115" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="13" t="inlineStr"/>
+      <c r="B116" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> ИТОГО докупка</t>
+        </is>
+      </c>
+      <c r="C116" s="13" t="inlineStr"/>
+      <c r="D116" s="13" t="n">
         <v>52</v>
       </c>
-      <c r="E95" s="13" t="inlineStr"/>
-    </row>
-    <row r="97">
-      <c r="A97" s="3" t="inlineStr">
-        <is>
-          <t>Тональный крем для лица матовый увлажняю</t>
-        </is>
-      </c>
-      <c r="B97" s="3" t="inlineStr">
+      <c r="E116" s="13" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="3" t="inlineStr">
+        <is>
+          <t>Сыворотка с микроиглами 1Dx для интенсив — ПЕРЕРАСПРЕДЕЛЕНИЕ (объёма хватает, развезти из Москвы)</t>
+        </is>
+      </c>
+      <c r="B118" s="3" t="inlineStr">
+        <is>
+          <t>Москва, МО и Дальние регионы</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="D118" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="E118" s="11" t="inlineStr">
+        <is>
+          <t>база, не перегружать</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="3" t="inlineStr"/>
+      <c r="B119" s="3" t="inlineStr">
+        <is>
+          <t>Санкт-Петербург и СЗО</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="D119" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E119" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="3" t="inlineStr"/>
+      <c r="B120" s="3" t="inlineStr">
+        <is>
+          <t>Дальний Восток</t>
+        </is>
+      </c>
+      <c r="C120" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D120" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E120" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="3" t="inlineStr"/>
+      <c r="B121" s="3" t="inlineStr">
+        <is>
+          <t>Воронеж</t>
+        </is>
+      </c>
+      <c r="C121" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D121" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E121" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="3" t="inlineStr"/>
+      <c r="B122" s="3" t="inlineStr">
+        <is>
+          <t>Саратов</t>
+        </is>
+      </c>
+      <c r="C122" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D122" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E122" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="3" t="inlineStr"/>
+      <c r="B123" s="3" t="inlineStr">
+        <is>
+          <t>Ярославль</t>
+        </is>
+      </c>
+      <c r="C123" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D123" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E123" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="3" t="inlineStr"/>
+      <c r="B124" s="3" t="inlineStr">
+        <is>
+          <t>Екатеринбург</t>
+        </is>
+      </c>
+      <c r="C124" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D124" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E124" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="3" t="inlineStr"/>
+      <c r="B125" s="3" t="inlineStr">
+        <is>
+          <t>Тверь</t>
+        </is>
+      </c>
+      <c r="C125" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D125" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E125" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="14" t="inlineStr"/>
+      <c r="B126" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> ИТОГО (перераспределение)</t>
+        </is>
+      </c>
+      <c r="C126" s="14" t="inlineStr"/>
+      <c r="D126" s="14" t="n">
+        <v>39</v>
+      </c>
+      <c r="E126" s="14" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="3" t="inlineStr">
+        <is>
+          <t>Отбеливающая сыворотка с ниацинамидом дл — ПЕРЕРАСПРЕДЕЛЕНИЕ (объёма хватает, развезти из Москвы)</t>
+        </is>
+      </c>
+      <c r="B128" s="3" t="inlineStr">
+        <is>
+          <t>Москва, МО и Дальние регионы</t>
+        </is>
+      </c>
+      <c r="C128" s="3" t="n">
+        <v>67</v>
+      </c>
+      <c r="D128" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="E128" s="11" t="inlineStr">
+        <is>
+          <t>база, не перегружать</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="3" t="inlineStr"/>
+      <c r="B129" s="3" t="inlineStr">
+        <is>
+          <t>Санкт-Петербург и СЗО</t>
+        </is>
+      </c>
+      <c r="C129" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="D129" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E129" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="3" t="inlineStr"/>
+      <c r="B130" s="3" t="inlineStr">
+        <is>
+          <t>Екатеринбург</t>
+        </is>
+      </c>
+      <c r="C130" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="D130" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E130" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="3" t="inlineStr"/>
+      <c r="B131" s="3" t="inlineStr">
+        <is>
+          <t>Ростов</t>
+        </is>
+      </c>
+      <c r="C131" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="D131" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E131" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="14" t="inlineStr"/>
+      <c r="B132" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> ИТОГО (перераспределение)</t>
+        </is>
+      </c>
+      <c r="C132" s="14" t="inlineStr"/>
+      <c r="D132" s="14" t="n">
+        <v>26</v>
+      </c>
+      <c r="E132" s="14" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="3" t="inlineStr">
+        <is>
+          <t>Восстанавливающая сыворотка для лица с б — ПЕРЕРАСПРЕДЕЛЕНИЕ (объёма хватает, развезти из Москвы)</t>
+        </is>
+      </c>
+      <c r="B134" s="3" t="inlineStr">
+        <is>
+          <t>Ростов</t>
+        </is>
+      </c>
+      <c r="C134" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="D134" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="E134" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="14" t="inlineStr"/>
+      <c r="B135" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> ИТОГО (перераспределение)</t>
+        </is>
+      </c>
+      <c r="C135" s="14" t="inlineStr"/>
+      <c r="D135" s="14" t="n">
+        <v>14</v>
+      </c>
+      <c r="E135" s="14" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="3" t="inlineStr">
+        <is>
+          <t>Гель пенка для умывания Bifida Complex A — ПЕРЕРАСПРЕДЕЛЕНИЕ (объёма хватает, развезти из Москвы)</t>
+        </is>
+      </c>
+      <c r="B137" s="3" t="inlineStr">
+        <is>
+          <t>Москва, МО и Дальние регионы</t>
+        </is>
+      </c>
+      <c r="C137" s="3" t="n">
+        <v>56</v>
+      </c>
+      <c r="D137" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E137" s="11" t="inlineStr">
+        <is>
+          <t>база, не перегружать</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="3" t="inlineStr"/>
+      <c r="B138" s="3" t="inlineStr">
+        <is>
+          <t>Санкт-Петербург и СЗО</t>
+        </is>
+      </c>
+      <c r="C138" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="D138" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E138" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="3" t="inlineStr"/>
+      <c r="B139" s="3" t="inlineStr">
+        <is>
+          <t>Тюмень</t>
+        </is>
+      </c>
+      <c r="C139" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D139" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E139" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="3" t="inlineStr"/>
+      <c r="B140" s="3" t="inlineStr">
+        <is>
+          <t>Саратов</t>
+        </is>
+      </c>
+      <c r="C140" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D140" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E140" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="14" t="inlineStr"/>
+      <c r="B141" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> ИТОГО (перераспределение)</t>
+        </is>
+      </c>
+      <c r="C141" s="14" t="inlineStr"/>
+      <c r="D141" s="14" t="n">
+        <v>13</v>
+      </c>
+      <c r="E141" s="14" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="3" t="inlineStr">
+        <is>
+          <t>Тональный крем для лица матирующий Colla — ДОКУПКА (не хватает на 45 дн)</t>
+        </is>
+      </c>
+      <c r="B143" s="3" t="inlineStr">
+        <is>
+          <t>Екатеринбург</t>
+        </is>
+      </c>
+      <c r="C143" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="D143" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E143" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="3" t="inlineStr"/>
+      <c r="B144" s="3" t="inlineStr">
+        <is>
+          <t>Ростов</t>
+        </is>
+      </c>
+      <c r="C144" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="D144" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E144" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="13" t="inlineStr"/>
+      <c r="B145" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> ИТОГО докупка</t>
+        </is>
+      </c>
+      <c r="C145" s="13" t="inlineStr"/>
+      <c r="D145" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="E145" s="13" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="3" t="inlineStr">
+        <is>
+          <t>Тональный крем для лица матирующий Colla — ПЕРЕРАСПРЕДЕЛЕНИЕ (объёма хватает, развезти из Москвы)</t>
+        </is>
+      </c>
+      <c r="B147" s="3" t="inlineStr">
+        <is>
+          <t>Санкт-Петербург и СЗО</t>
+        </is>
+      </c>
+      <c r="C147" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="D147" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E147" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="3" t="inlineStr"/>
+      <c r="B148" s="3" t="inlineStr">
+        <is>
+          <t>Москва, МО и Дальние регионы</t>
+        </is>
+      </c>
+      <c r="C148" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="D148" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E148" s="11" t="inlineStr">
+        <is>
+          <t>база, не перегружать</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="3" t="inlineStr"/>
+      <c r="B149" s="3" t="inlineStr">
+        <is>
+          <t>Оренбург</t>
+        </is>
+      </c>
+      <c r="C149" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="D149" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E149" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="14" t="inlineStr"/>
+      <c r="B150" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> ИТОГО (перераспределение)</t>
+        </is>
+      </c>
+      <c r="C150" s="14" t="inlineStr"/>
+      <c r="D150" s="14" t="n">
+        <v>13</v>
+      </c>
+      <c r="E150" s="14" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="3" t="inlineStr">
+        <is>
+          <t>Тональный крем для лица матовый увлажняю — ДОКУПКА (не хватает на 45 дн)</t>
+        </is>
+      </c>
+      <c r="B152" s="3" t="inlineStr">
         <is>
           <t>Уфа</t>
         </is>
       </c>
-      <c r="C97" s="3" t="n">
+      <c r="C152" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="D97" s="3" t="n">
+      <c r="D152" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="E97" s="12" t="inlineStr">
-        <is>
-          <t>грузить</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="3" t="inlineStr"/>
-      <c r="B98" s="3" t="inlineStr">
+      <c r="E152" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="3" t="inlineStr"/>
+      <c r="B153" s="3" t="inlineStr">
         <is>
           <t>Красноярск</t>
         </is>
       </c>
-      <c r="C98" s="3" t="n">
+      <c r="C153" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="D98" s="3" t="n">
+      <c r="D153" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="E98" s="12" t="inlineStr">
-        <is>
-          <t>грузить</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="13" t="inlineStr"/>
-      <c r="B99" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> ИТОГО</t>
-        </is>
-      </c>
-      <c r="C99" s="13" t="inlineStr"/>
-      <c r="D99" s="13" t="n">
+      <c r="E153" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="13" t="inlineStr"/>
+      <c r="B154" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> ИТОГО докупка</t>
+        </is>
+      </c>
+      <c r="C154" s="13" t="inlineStr"/>
+      <c r="D154" s="13" t="n">
         <v>13</v>
       </c>
-      <c r="E99" s="13" t="inlineStr"/>
+      <c r="E154" s="13" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="3" t="inlineStr">
+        <is>
+          <t>Лосьон для лица Bifida Biome Ampoule Lot — ПЕРЕРАСПРЕДЕЛЕНИЕ (объёма хватает, развезти из Москвы) (общая доля магазина)</t>
+        </is>
+      </c>
+      <c r="B156" s="3" t="inlineStr">
+        <is>
+          <t>Москва, МО и Дальние регионы</t>
+        </is>
+      </c>
+      <c r="C156" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="D156" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E156" s="11" t="inlineStr">
+        <is>
+          <t>база, не перегружать</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="3" t="inlineStr"/>
+      <c r="B157" s="3" t="inlineStr">
+        <is>
+          <t>Санкт-Петербург и СЗО</t>
+        </is>
+      </c>
+      <c r="C157" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="D157" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E157" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="3" t="inlineStr"/>
+      <c r="B158" s="3" t="inlineStr">
+        <is>
+          <t>Ростов</t>
+        </is>
+      </c>
+      <c r="C158" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="D158" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E158" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="3" t="inlineStr"/>
+      <c r="B159" s="3" t="inlineStr">
+        <is>
+          <t>Казань</t>
+        </is>
+      </c>
+      <c r="C159" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D159" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E159" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="3" t="inlineStr"/>
+      <c r="B160" s="3" t="inlineStr">
+        <is>
+          <t>Воронеж</t>
+        </is>
+      </c>
+      <c r="C160" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D160" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E160" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="3" t="inlineStr"/>
+      <c r="B161" s="3" t="inlineStr">
+        <is>
+          <t>Краснодар</t>
+        </is>
+      </c>
+      <c r="C161" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D161" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E161" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="3" t="inlineStr"/>
+      <c r="B162" s="3" t="inlineStr">
+        <is>
+          <t>Дальний Восток</t>
+        </is>
+      </c>
+      <c r="C162" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D162" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E162" s="12" t="inlineStr">
+        <is>
+          <t>грузить</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="14" t="inlineStr"/>
+      <c r="B163" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> ИТОГО (перераспределение)</t>
+        </is>
+      </c>
+      <c r="C163" s="14" t="inlineStr"/>
+      <c r="D163" s="14" t="n">
+        <v>13</v>
+      </c>
+      <c r="E163" s="14" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>